<commit_message>
Feat: Updated containerization and improved  csv files that are incomplete
</commit_message>
<xml_diff>
--- a/main/data/MyCandidate Seed Doc.xlsx
+++ b/main/data/MyCandidate Seed Doc.xlsx
@@ -1,25 +1,29 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" mc:Ignorable="x15">
-  <fileVersion appName="xl" lastEdited="6" lowestEdited="6" rupBuild="14420"/>
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="29127"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Projects\OCL\mycandidate\main\data\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Coding\mycandidate\main\data\"/>
     </mc:Choice>
   </mc:AlternateContent>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{89CCF827-5002-4BD1-805D-C113DDC1BBD0}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="0" windowWidth="20490" windowHeight="7620"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="16440" activeTab="3" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="site_settings" sheetId="1" r:id="rId1"/>
+    <sheet name="Provincial" sheetId="2" r:id="rId2"/>
+    <sheet name="National" sheetId="3" r:id="rId3"/>
+    <sheet name="Regional" sheetId="4" r:id="rId4"/>
   </sheets>
   <calcPr calcId="0"/>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="38" uniqueCount="38">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="98" uniqueCount="38">
   <si>
     <t>title</t>
   </si>
@@ -143,7 +147,7 @@
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
-<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" mc:Ignorable="x14ac x16r2">
+<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
   <fonts count="4" x14ac:knownFonts="1">
     <font>
       <sz val="10"/>
@@ -211,7 +215,7 @@
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
   <cellXfs count="4">
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
@@ -436,7 +440,7 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <sheetPr>
     <outlinePr summaryBelow="0" summaryRight="0"/>
   </sheetPr>
@@ -586,9 +590,237 @@
     </row>
   </sheetData>
   <hyperlinks>
-    <hyperlink ref="F2" r:id="rId1" display="http://opencitieslab.org/"/>
+    <hyperlink ref="F2" r:id="rId1" display="http://opencitieslab.org/" xr:uid="{00000000-0004-0000-0000-000000000000}"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup paperSize="9" orientation="portrait" r:id="rId2"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{A8B5BC3E-EFB2-4785-BF33-F5FB388B848F}">
+  <dimension ref="A1:K2"/>
+  <sheetFormatPr defaultColWidth="24.5703125" defaultRowHeight="12.75" x14ac:dyDescent="0.2"/>
+  <sheetData>
+    <row r="1" spans="1:11" ht="13.5" thickBot="1" x14ac:dyDescent="0.25">
+      <c r="A1" s="1" t="s">
+        <v>13</v>
+      </c>
+      <c r="B1" s="1" t="s">
+        <v>14</v>
+      </c>
+      <c r="C1" s="1" t="s">
+        <v>15</v>
+      </c>
+      <c r="D1" s="1" t="s">
+        <v>16</v>
+      </c>
+      <c r="E1" s="1" t="s">
+        <v>17</v>
+      </c>
+      <c r="F1" s="1" t="s">
+        <v>18</v>
+      </c>
+      <c r="G1" s="1" t="s">
+        <v>25</v>
+      </c>
+      <c r="H1" s="1" t="s">
+        <v>26</v>
+      </c>
+      <c r="I1" s="1" t="s">
+        <v>27</v>
+      </c>
+      <c r="J1" s="1" t="s">
+        <v>28</v>
+      </c>
+      <c r="K1" s="1"/>
+    </row>
+    <row r="2" spans="1:11" ht="204.75" thickBot="1" x14ac:dyDescent="0.25">
+      <c r="A2" s="1" t="s">
+        <v>19</v>
+      </c>
+      <c r="B2" s="1" t="s">
+        <v>20</v>
+      </c>
+      <c r="C2" s="1" t="s">
+        <v>21</v>
+      </c>
+      <c r="D2" s="1" t="s">
+        <v>22</v>
+      </c>
+      <c r="E2" s="1" t="s">
+        <v>23</v>
+      </c>
+      <c r="F2" s="1" t="s">
+        <v>24</v>
+      </c>
+      <c r="G2" s="1" t="s">
+        <v>32</v>
+      </c>
+      <c r="H2" s="1" t="s">
+        <v>35</v>
+      </c>
+      <c r="I2" s="1" t="s">
+        <v>36</v>
+      </c>
+      <c r="J2" s="1" t="s">
+        <v>37</v>
+      </c>
+      <c r="K2" s="1"/>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{983F7C53-9B4E-4F64-AEAA-D883EED29D79}">
+  <dimension ref="A1:K2"/>
+  <sheetFormatPr defaultRowHeight="12.75" x14ac:dyDescent="0.2"/>
+  <sheetData>
+    <row r="1" spans="1:11" ht="39" thickBot="1" x14ac:dyDescent="0.25">
+      <c r="A1" s="1" t="s">
+        <v>13</v>
+      </c>
+      <c r="B1" s="1" t="s">
+        <v>14</v>
+      </c>
+      <c r="C1" s="1" t="s">
+        <v>15</v>
+      </c>
+      <c r="D1" s="1" t="s">
+        <v>16</v>
+      </c>
+      <c r="E1" s="1" t="s">
+        <v>17</v>
+      </c>
+      <c r="F1" s="1" t="s">
+        <v>18</v>
+      </c>
+      <c r="G1" s="1" t="s">
+        <v>25</v>
+      </c>
+      <c r="H1" s="1" t="s">
+        <v>26</v>
+      </c>
+      <c r="I1" s="1" t="s">
+        <v>27</v>
+      </c>
+      <c r="J1" s="1" t="s">
+        <v>28</v>
+      </c>
+      <c r="K1" s="1"/>
+    </row>
+    <row r="2" spans="1:11" ht="204.75" thickBot="1" x14ac:dyDescent="0.25">
+      <c r="A2" s="1" t="s">
+        <v>19</v>
+      </c>
+      <c r="B2" s="1" t="s">
+        <v>20</v>
+      </c>
+      <c r="C2" s="1" t="s">
+        <v>21</v>
+      </c>
+      <c r="D2" s="1" t="s">
+        <v>22</v>
+      </c>
+      <c r="E2" s="1" t="s">
+        <v>23</v>
+      </c>
+      <c r="F2" s="1" t="s">
+        <v>24</v>
+      </c>
+      <c r="G2" s="1" t="s">
+        <v>32</v>
+      </c>
+      <c r="H2" s="1" t="s">
+        <v>35</v>
+      </c>
+      <c r="I2" s="1" t="s">
+        <v>36</v>
+      </c>
+      <c r="J2" s="1" t="s">
+        <v>37</v>
+      </c>
+      <c r="K2" s="1"/>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{A4C24526-2D37-4DD4-AC78-7CA5606DEE9C}">
+  <dimension ref="A1:K2"/>
+  <sheetFormatPr defaultRowHeight="12.75" x14ac:dyDescent="0.2"/>
+  <sheetData>
+    <row r="1" spans="1:11" ht="39" thickBot="1" x14ac:dyDescent="0.25">
+      <c r="A1" s="1" t="s">
+        <v>13</v>
+      </c>
+      <c r="B1" s="1" t="s">
+        <v>14</v>
+      </c>
+      <c r="C1" s="1" t="s">
+        <v>15</v>
+      </c>
+      <c r="D1" s="1" t="s">
+        <v>16</v>
+      </c>
+      <c r="E1" s="1" t="s">
+        <v>17</v>
+      </c>
+      <c r="F1" s="1" t="s">
+        <v>18</v>
+      </c>
+      <c r="G1" s="1" t="s">
+        <v>25</v>
+      </c>
+      <c r="H1" s="1" t="s">
+        <v>26</v>
+      </c>
+      <c r="I1" s="1" t="s">
+        <v>27</v>
+      </c>
+      <c r="J1" s="1" t="s">
+        <v>28</v>
+      </c>
+      <c r="K1" s="1"/>
+    </row>
+    <row r="2" spans="1:11" ht="204.75" thickBot="1" x14ac:dyDescent="0.25">
+      <c r="A2" s="1" t="s">
+        <v>19</v>
+      </c>
+      <c r="B2" s="1" t="s">
+        <v>20</v>
+      </c>
+      <c r="C2" s="1" t="s">
+        <v>21</v>
+      </c>
+      <c r="D2" s="1" t="s">
+        <v>22</v>
+      </c>
+      <c r="E2" s="1" t="s">
+        <v>23</v>
+      </c>
+      <c r="F2" s="1" t="s">
+        <v>24</v>
+      </c>
+      <c r="G2" s="1" t="s">
+        <v>32</v>
+      </c>
+      <c r="H2" s="1" t="s">
+        <v>35</v>
+      </c>
+      <c r="I2" s="1" t="s">
+        <v>36</v>
+      </c>
+      <c r="J2" s="1" t="s">
+        <v>37</v>
+      </c>
+      <c r="K2" s="1"/>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
 </file>
</xml_diff>